<commit_message>
corpus(s53): base instalada TRATEIN (multi-marca, vía /my-orders) — inventario 4 marcas (DEC-029)
- 76 PDFs de los 41 productos comprados (10 pedidos TRATEIN PCI), agrupados por
  marca real: Kidde (devices) / Aritech / Edwards / Otros (genéricos sin marca).
- Método nuevo (orders -> order_details -> line_items -> product_downloads),
  reproducible en docs/CORPUS_FIRESECURITYPRODUCTS.md §7.
- Inventario 4 marcas: Kidde 33/55, Aritech 13/33, Edwards 2/3, Otros 12/16.
- update_inventario.py: +3 entradas FABRICANTES; .gitignore: 3 carpetas ignoradas.
- Parse LlamaParse lanzado (~66 ficheros/893pp/~$50); verificacion pendiente.
- INERTE al corpus/eval: ingesta a chunks_v2 DIFERIDA (gate RULER + Protocolo 3).
- 2X-A cross-listed Kidde(s52)/Aritech(OEM): el portal cross-brandea (documentado).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Inventario_Manuales.xlsx
+++ b/data/Inventario_Manuales.xlsx
@@ -12,6 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Morley" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notifier" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kidde" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aritech" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edwards" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Otros" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -514,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -642,17 +645,110 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="C11" t="n">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Portal firesecurityproducts (paneles Control · ES+EN)</t>
-        </is>
-      </c>
-    </row>
+          <t>Portal firesecurityproducts — paneles Control (s52) + base instalada TRATEIN (Excellence/ModuLaser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Aritech</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>13</v>
+      </c>
+      <c r="C12" t="n">
+        <v>33</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Portal firesecurityproducts — base instalada TRATEIN (paneles 2X-A, detección serie 2000, módulos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Edwards</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Portal firesecurityproducts — base instalada TRATEIN (ModuLaser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>12</v>
+      </c>
+      <c r="C14" t="n">
+        <v>16</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Portal firesecurityproducts — base instalada TRATEIN (genéricos sin marca: tubería, cable, accesorios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
@@ -34169,7 +34265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -34455,12 +34551,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2X-AF1-S</t>
+          <t>KE-DM3010R-KIT</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Datasheet</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -34475,17 +34571,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2x-af1-s-161721-es.pdf</t>
+          <t>03-0210-501-4300-06_r006_excellence_series_addressable_mcp_installation_sheet_ml.pdf</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>890</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2X-AF2-FB</t>
+          <t>2X-AF1-S</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -34505,17 +34601,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2x-af2-fb-161721-es.pdf</t>
+          <t>2x-af1-s-161721-es.pdf</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1101</v>
+        <v>890</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2X-AF2-FB-S</t>
+          <t>2X-AF2-FB</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -34535,17 +34631,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2x-af2-fb-s-161721-es.pdf</t>
+          <t>2x-af2-fb-161721-es.pdf</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>952</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2X-AF2-SCFB</t>
+          <t>2X-AF2-FB-S</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -34565,17 +34661,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2x-af2-scfb-161721-es.pdf</t>
+          <t>2x-af2-fb-s-161721-es.pdf</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1090</v>
+        <v>952</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2X-AF2-SCFB-S</t>
+          <t>2X-AF2-SCFB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -34595,17 +34691,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2x-af2-scfb-s-161721-es.pdf</t>
+          <t>2x-af2-scfb-161721-es.pdf</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>903</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2X-AT-F2</t>
+          <t>2X-AF2-SCFB-S</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -34625,17 +34721,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2x-at-f2-161721-es.pdf</t>
+          <t>2x-af2-scfb-s-161721-es.pdf</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>497</v>
+        <v>903</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2X-AT-F2-FB</t>
+          <t>2X-AT-F2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -34655,17 +34751,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2x-at-f2-fb-161721-es.pdf</t>
+          <t>2x-at-f2-161721-es.pdf</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>473</v>
+        <v>497</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2X-AT-F2-FB-P</t>
+          <t>2X-AT-F2-FB</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -34685,17 +34781,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2x-at-f2-fb-p-161721-es.pdf</t>
+          <t>2x-at-f2-fb-161721-es.pdf</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2X-AT-F2-FB-S</t>
+          <t>2X-AT-F2-FB-P</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -34715,17 +34811,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2x-at-f2-fb-s-161721-es.pdf</t>
+          <t>2x-at-f2-fb-p-161721-es.pdf</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>339</v>
+        <v>472</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2X-AT-F2-P</t>
+          <t>2X-AT-F2-FB-S</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -34745,17 +34841,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2x-at-f2-p-161721-es.pdf</t>
+          <t>2x-at-f2-fb-s-161721-es.pdf</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>473</v>
+        <v>339</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2X-AT-F2-S</t>
+          <t>2X-AT-F2-P</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -34775,27 +34871,27 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2x-at-f2-s-161721-es.pdf</t>
+          <t>2x-at-f2-p-161721-es.pdf</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>523</v>
+        <v>473</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2X-A Táctil</t>
+          <t>2X-AT-F2-S</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Manual técnico</t>
+          <t>Datasheet</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -34805,17 +34901,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>3103267-en_r001_2x-a_series_kuwait_marketplace_manual.pdf</t>
+          <t>2x-at-f2-s-161721-es.pdf</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>355</v>
+        <v>523</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>KE-DP3020W</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -34835,22 +34931,22 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>bcn-3100017-es_r002_nc_series_fire_alarm_control_panel_installation_manual.pdf</t>
+          <t>3102984-ml_r003_excellence_series_intelligent_addressable_dual_optical_detector_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>3723</v>
+        <v>716</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>KE-DT3001W-HAB</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Manual usuario</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -34865,22 +34961,22 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>bcn-3100018-es_r002_nc_series_fire_alarm_control_panel_operation_manual.pdf</t>
+          <t>3102986-ml_r002_excellence_series_intelligent_addressable_class_a-b_heat_detector_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>767</v>
+        <v>724</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>KE-DB3010W</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Guía rápida</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -34895,22 +34991,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>bcn-3100019-es_r002_nc_series_fire_alarm_control_panel_quick_installation_guide.pdf</t>
+          <t>3102987-ml_r003_excellence_series_standard_mounting_base_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>323</v>
+        <v>659</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>KE-DBA-AUXW</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Guía rápida</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -34925,27 +35021,27 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>bcn-3100020-es_r002_nc_series_fire_alarm_control_panel_quick_operation_guide.pdf</t>
+          <t>3103013-ml_r002_ke-dba-auxw_deep_accessory_for_standard_mounting_base_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>222</v>
+        <v>780</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2X-A Táctil</t>
+          <t>KE-IO3101</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Manual técnico</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -34955,27 +35051,27 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>bcn-3100035-en_r006_2x-a_series_addressable_control_panel_compatibility_list_0.pdf</t>
+          <t>3103062-ml_r003_excellence_series_addressable_single_output_module_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>215</v>
+        <v>636</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2X-A Táctil</t>
+          <t>KE-IO3122</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Manual técnico</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -34985,22 +35081,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>bcn-3100036-en_r002_2x-a_and_zp2-a_series_addressable_control_panel_compatibility_list_900_series_protocol.pdf</t>
+          <t>3103063-ml_r003_excellence_series_addressable_two-four_input-output_module_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>193</v>
+        <v>839</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>NC-PF2</t>
+          <t>KE-AS3115R-WM</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Datasheet</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -35015,22 +35111,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>nc-pf2-161721-es.pdf</t>
+          <t>3103072-ml_r004_excellence_series_intelligent_addressable_indoor_notification_device_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>497</v>
+        <v>3036</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>NC-PF4</t>
+          <t>9-30781-KID-EN</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Datasheet</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -35045,22 +35141,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>nc-pf4-161721-es.pdf</t>
+          <t>3103092-es_r003_modulaser_en_54-20_installation_manual_kidde_0.pdf</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>622</v>
+        <v>6029</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>NC-PF4-SC</t>
+          <t>KE-AS3115R-WMIP</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Datasheet</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -35075,27 +35171,27 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>nc-pf4-sc-161721-es.pdf</t>
+          <t>3103198-ml_r002_excellence_series_intelligent_addressable_outdoor_notification_device_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>628</v>
+        <v>3366</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NC-PF8</t>
+          <t>2X-A Táctil</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Datasheet</t>
+          <t>Manual técnico</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>EN</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -35105,19 +35201,1723 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>nc-pf8-161721-es.pdf</t>
+          <t>3103267-en_r001_2x-a_series_kuwait_marketplace_manual.pdf</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>560</v>
+        <v>355</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>9-30781-KID-EN</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>9-30781-kid-en-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>9-30783-KID-EN</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>9-30783-kid-en-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>bcn-3100017-es_r002_nc_series_fire_alarm_control_panel_installation_manual.pdf</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>3723</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Manual usuario</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>bcn-3100018-es_r002_nc_series_fire_alarm_control_panel_operation_manual.pdf</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>bcn-3100019-es_r002_nc_series_fire_alarm_control_panel_quick_installation_guide.pdf</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>bcn-3100020-es_r002_nc_series_fire_alarm_control_panel_quick_operation_guide.pdf</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2X-A Táctil</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>bcn-3100035-en_r006_2x-a_series_addressable_control_panel_compatibility_list_0.pdf</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2X-A Táctil</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>bcn-3100036-en_r002_2x-a_and_zp2-a_series_addressable_control_panel_compatibility_list_900_series_protocol.pdf</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>KE-AS3115R-WM</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ke-as3115r-wm-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>KE-AS3115R-WMIP</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ke-as3115r-wmip-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>KE-DB3010W</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ke-db3010w-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KE-DBA-AUXW</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ke-dba-auxw-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>KE-DM3010R</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ke-dm3010r-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>KE-DM3010R-KIT</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ke-dm3010r-kit-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>KE-DP3020W</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ke-dp3020w-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>KE-DP3120W</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>ke-dp3120w-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>KE-DT3001W-HAB</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ke-dt3001w-hab-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>KE-IO3101</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ke-io3101-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>KE-IO3122</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ke-io3122-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>KE-IO3144</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ke-io3144-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>NC-PF2</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>nc-pf2-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>NC-PF4</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>nc-pf4-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>NC-PF4-SC</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>nc-pf4-sc-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>NC-PF8</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>nc-pf8-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>NC-PF8-SC</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>nc-pf8-sc-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>617</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Tipo documento</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Idioma</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Subcarpeta</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Archivo</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Tamaño (KB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2X-LB</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>00-3218-501-0000-07_r007_2x-lb_installation_sheet_ml.pdf</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>00-3280-501-4003-05_r005_2x-a_series_installation_manual_en_0.pdf</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>4810</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2X-AF2-09</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>00-3280-501-4009-05_r005_2x-a_series_installation_manual_es.pdf</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>5001</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2X-AF2-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Manual usuario</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>00-3280-505-4009-04_r004_2x-a_series_operation_manual_es.pdf</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>00-3280-507-4003-03_r003_2x-a_series_quick_installation_guide_en.pdf</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2X-AF2-09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>00-3280-507-4009-03_r003_2x-a_series_quick_installation_guide_es.pdf</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2X-AF2-09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>00-3280-508-4009-03_r003_2x-a_series_quick_operation_guide_es.pdf</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>00-3280-508-4109-06_r006_2x-at_series_quick_start_guide_es.pdf</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>00-3280-508-4209-02_r002_2x-at_series_quick_operation_guide_es.pdf</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2X-A-LB</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>00-3301-501-4000-04_r004_2x-a-lb_loop_board_installation_sheet_ml.pdf</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2010-2A-PAK-HPL</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>00-3301-501-4100-04_r004_2010-2a-pak-hpl_registration_guide_ml.pdf</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>FD2705R</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0044-055-02_-_aritech_ra_-_fd2705-10r_addendum_-_en_de.pdf</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>IU2055NC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>10-5106-501-55nc-05_r005_iu2055nc_installation_sheet_ml.pdf</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AS2364</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>18-187110-10.pdf</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1608</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2010-2-PAK-RMSDK</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2010-2-pak-rmsdk-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2010-2A-PAK-HPL</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2010-2a-pak-hpl-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>FD2705R</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Manual usuario</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>22318.18.08_-_aritech_ra_-_fd2705-10r_english_std_reflective_user_guide_-_en.pdf</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2X-A-LB</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2x-a-lb-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1557</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2X-AF2-09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2x-af2-09-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2x-at-f2-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2X-LB</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2x-lb-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1556</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>3103267-en_r001_2x-a_series_kuwait_marketplace_manual.pdf</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ASW2367</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>aritech_ins570-8_combined.pdf</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>AS2363</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>as2363-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>AS2364</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>as2364-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ASW2366</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>asw2366-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ASW2367</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>asw2367-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2010-2-PAK-RMSDK</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>bcn-3100032-ml_r002_2010-2-pak-rmsdk_registration_guide.pdf</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>bcn-3100035-en_r006_2x-a_series_addressable_control_panel_compatibility_list_0.pdf</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>bcn-3100036-en_r002_2x-a_and_zp2-a_series_addressable_control_panel_compatibility_list_900_series_protocol.pdf</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>FD2705R</t>
+        </is>
+      </c>
       <c r="B32" t="inlineStr">
         <is>
           <t>Datasheet</t>
@@ -35135,11 +36935,749 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>nc-pf8-sc-161721-es.pdf</t>
+          <t>fd2705r-62536-es.pdf</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>617</v>
+        <v>499</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FD2710R</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>fd2710r-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>IU2055NC</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>iu2055nc-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1069</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Tipo documento</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Idioma</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Subcarpeta</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Archivo</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Tamaño (KB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FHSD8310</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>04-4001-501-2009-12_r012_modulaser_en_54-20_installation_manual_es_edwards_0.pdf</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>6021</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FHSD8310</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>fhsd8310-63296-es.pdf</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FHSD8330</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>fhsd8330-63296-es.pdf</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>462</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Tipo documento</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Idioma</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Subcarpeta</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Archivo</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Tamaño (KB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>N-MC-BB-G</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>03-0210-501-4301-02_r002_n-mc_series_mcp_backbox_installation_sheet_ml.pdf</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NC-MC-0-G</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>03-0211-501-3000-05_r005_nc_series_conventional_mcp_installation_sheet_ml_0.pdf</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>9-30441</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>04-4001-501-1700-06_r006_aritech_apic_installation_sheet_ml_0.pdf</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AD68N-0100</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>20-8501-509-dl03-04_alarmline_ii_digital_lhd_cable_technical_manual_en.pdf</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>9-10900</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>9-10900-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>9-10906</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>9-10906-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9-10908</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>9-10908-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9-10909</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>9-10909-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>9-10927</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>9-10927-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>9-10954-100</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>9-10954-100-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9-30441</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>9-30441-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AD68N-0100</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ad68n-0100-1-es.pdf</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DM715</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>dm715-63296-es.pdf</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>N-MC-BB-G</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>n-mc-bb-g-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NC-MC-0-G</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nc-mc-0-g-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SC010</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>sds0098es_solo_a10_iss_2.1.pdf</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
corpus(s53): base instalada TRATEIN (multi-marca, vía /my-orders) — inventario 4 marcas (DEC-029) (#47)
- 76 PDFs de los 41 productos comprados (10 pedidos TRATEIN PCI), agrupados por
  marca real: Kidde (devices) / Aritech / Edwards / Otros (genéricos sin marca).
- Método nuevo (orders -> order_details -> line_items -> product_downloads),
  reproducible en docs/CORPUS_FIRESECURITYPRODUCTS.md §7.
- Inventario 4 marcas: Kidde 33/55, Aritech 13/33, Edwards 2/3, Otros 12/16.
- update_inventario.py: +3 entradas FABRICANTES; .gitignore: 3 carpetas ignoradas.
- Parse LlamaParse lanzado (~66 ficheros/893pp/~$50); verificacion pendiente.
- INERTE al corpus/eval: ingesta a chunks_v2 DIFERIDA (gate RULER + Protocolo 3).
- 2X-A cross-listed Kidde(s52)/Aritech(OEM): el portal cross-brandea (documentado).

Co-authored-by: albertofontiber <271603099+albertofontiber@users.noreply.github.com>
Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Inventario_Manuales.xlsx
+++ b/data/Inventario_Manuales.xlsx
@@ -12,6 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Morley" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notifier" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kidde" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aritech" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edwards" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Otros" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -514,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -642,17 +645,110 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="C11" t="n">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Portal firesecurityproducts (paneles Control · ES+EN)</t>
-        </is>
-      </c>
-    </row>
+          <t>Portal firesecurityproducts — paneles Control (s52) + base instalada TRATEIN (Excellence/ModuLaser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Aritech</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>13</v>
+      </c>
+      <c r="C12" t="n">
+        <v>33</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Portal firesecurityproducts — base instalada TRATEIN (paneles 2X-A, detección serie 2000, módulos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Edwards</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Portal firesecurityproducts — base instalada TRATEIN (ModuLaser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>12</v>
+      </c>
+      <c r="C14" t="n">
+        <v>16</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Portal firesecurityproducts — base instalada TRATEIN (genéricos sin marca: tubería, cable, accesorios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
@@ -34169,7 +34265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -34455,12 +34551,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2X-AF1-S</t>
+          <t>KE-DM3010R-KIT</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Datasheet</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -34475,17 +34571,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2x-af1-s-161721-es.pdf</t>
+          <t>03-0210-501-4300-06_r006_excellence_series_addressable_mcp_installation_sheet_ml.pdf</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>890</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2X-AF2-FB</t>
+          <t>2X-AF1-S</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -34505,17 +34601,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2x-af2-fb-161721-es.pdf</t>
+          <t>2x-af1-s-161721-es.pdf</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1101</v>
+        <v>890</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2X-AF2-FB-S</t>
+          <t>2X-AF2-FB</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -34535,17 +34631,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2x-af2-fb-s-161721-es.pdf</t>
+          <t>2x-af2-fb-161721-es.pdf</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>952</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2X-AF2-SCFB</t>
+          <t>2X-AF2-FB-S</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -34565,17 +34661,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2x-af2-scfb-161721-es.pdf</t>
+          <t>2x-af2-fb-s-161721-es.pdf</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1090</v>
+        <v>952</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2X-AF2-SCFB-S</t>
+          <t>2X-AF2-SCFB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -34595,17 +34691,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2x-af2-scfb-s-161721-es.pdf</t>
+          <t>2x-af2-scfb-161721-es.pdf</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>903</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2X-AT-F2</t>
+          <t>2X-AF2-SCFB-S</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -34625,17 +34721,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2x-at-f2-161721-es.pdf</t>
+          <t>2x-af2-scfb-s-161721-es.pdf</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>497</v>
+        <v>903</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2X-AT-F2-FB</t>
+          <t>2X-AT-F2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -34655,17 +34751,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2x-at-f2-fb-161721-es.pdf</t>
+          <t>2x-at-f2-161721-es.pdf</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>473</v>
+        <v>497</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2X-AT-F2-FB-P</t>
+          <t>2X-AT-F2-FB</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -34685,17 +34781,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2x-at-f2-fb-p-161721-es.pdf</t>
+          <t>2x-at-f2-fb-161721-es.pdf</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2X-AT-F2-FB-S</t>
+          <t>2X-AT-F2-FB-P</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -34715,17 +34811,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2x-at-f2-fb-s-161721-es.pdf</t>
+          <t>2x-at-f2-fb-p-161721-es.pdf</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>339</v>
+        <v>472</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2X-AT-F2-P</t>
+          <t>2X-AT-F2-FB-S</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -34745,17 +34841,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2x-at-f2-p-161721-es.pdf</t>
+          <t>2x-at-f2-fb-s-161721-es.pdf</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>473</v>
+        <v>339</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2X-AT-F2-S</t>
+          <t>2X-AT-F2-P</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -34775,27 +34871,27 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2x-at-f2-s-161721-es.pdf</t>
+          <t>2x-at-f2-p-161721-es.pdf</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>523</v>
+        <v>473</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2X-A Táctil</t>
+          <t>2X-AT-F2-S</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Manual técnico</t>
+          <t>Datasheet</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -34805,17 +34901,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>3103267-en_r001_2x-a_series_kuwait_marketplace_manual.pdf</t>
+          <t>2x-at-f2-s-161721-es.pdf</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>355</v>
+        <v>523</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>KE-DP3020W</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -34835,22 +34931,22 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>bcn-3100017-es_r002_nc_series_fire_alarm_control_panel_installation_manual.pdf</t>
+          <t>3102984-ml_r003_excellence_series_intelligent_addressable_dual_optical_detector_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>3723</v>
+        <v>716</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>KE-DT3001W-HAB</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Manual usuario</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -34865,22 +34961,22 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>bcn-3100018-es_r002_nc_series_fire_alarm_control_panel_operation_manual.pdf</t>
+          <t>3102986-ml_r002_excellence_series_intelligent_addressable_class_a-b_heat_detector_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>767</v>
+        <v>724</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>KE-DB3010W</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Guía rápida</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -34895,22 +34991,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>bcn-3100019-es_r002_nc_series_fire_alarm_control_panel_quick_installation_guide.pdf</t>
+          <t>3102987-ml_r003_excellence_series_standard_mounting_base_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>323</v>
+        <v>659</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>KE-DBA-AUXW</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Guía rápida</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -34925,27 +35021,27 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>bcn-3100020-es_r002_nc_series_fire_alarm_control_panel_quick_operation_guide.pdf</t>
+          <t>3103013-ml_r002_ke-dba-auxw_deep_accessory_for_standard_mounting_base_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>222</v>
+        <v>780</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2X-A Táctil</t>
+          <t>KE-IO3101</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Manual técnico</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -34955,27 +35051,27 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>bcn-3100035-en_r006_2x-a_series_addressable_control_panel_compatibility_list_0.pdf</t>
+          <t>3103062-ml_r003_excellence_series_addressable_single_output_module_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>215</v>
+        <v>636</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2X-A Táctil</t>
+          <t>KE-IO3122</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Manual técnico</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -34985,22 +35081,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>bcn-3100036-en_r002_2x-a_and_zp2-a_series_addressable_control_panel_compatibility_list_900_series_protocol.pdf</t>
+          <t>3103063-ml_r003_excellence_series_addressable_two-four_input-output_module_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>193</v>
+        <v>839</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>NC-PF2</t>
+          <t>KE-AS3115R-WM</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Datasheet</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -35015,22 +35111,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>nc-pf2-161721-es.pdf</t>
+          <t>3103072-ml_r004_excellence_series_intelligent_addressable_indoor_notification_device_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>497</v>
+        <v>3036</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>NC-PF4</t>
+          <t>9-30781-KID-EN</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Datasheet</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -35045,22 +35141,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>nc-pf4-161721-es.pdf</t>
+          <t>3103092-es_r003_modulaser_en_54-20_installation_manual_kidde_0.pdf</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>622</v>
+        <v>6029</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>NC-PF4-SC</t>
+          <t>KE-AS3115R-WMIP</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Datasheet</t>
+          <t>Manual instalación</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -35075,27 +35171,27 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>nc-pf4-sc-161721-es.pdf</t>
+          <t>3103198-ml_r002_excellence_series_intelligent_addressable_outdoor_notification_device_installation_sheet.pdf</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>628</v>
+        <v>3366</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NC-PF8</t>
+          <t>2X-A Táctil</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Datasheet</t>
+          <t>Manual técnico</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>EN</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -35105,19 +35201,1723 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>nc-pf8-161721-es.pdf</t>
+          <t>3103267-en_r001_2x-a_series_kuwait_marketplace_manual.pdf</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>560</v>
+        <v>355</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>9-30781-KID-EN</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>9-30781-kid-en-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>9-30783-KID-EN</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>9-30783-kid-en-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>bcn-3100017-es_r002_nc_series_fire_alarm_control_panel_installation_manual.pdf</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>3723</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Manual usuario</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>bcn-3100018-es_r002_nc_series_fire_alarm_control_panel_operation_manual.pdf</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>bcn-3100019-es_r002_nc_series_fire_alarm_control_panel_quick_installation_guide.pdf</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>bcn-3100020-es_r002_nc_series_fire_alarm_control_panel_quick_operation_guide.pdf</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2X-A Táctil</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>bcn-3100035-en_r006_2x-a_series_addressable_control_panel_compatibility_list_0.pdf</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2X-A Táctil</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>bcn-3100036-en_r002_2x-a_and_zp2-a_series_addressable_control_panel_compatibility_list_900_series_protocol.pdf</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>KE-AS3115R-WM</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ke-as3115r-wm-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>KE-AS3115R-WMIP</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ke-as3115r-wmip-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>KE-DB3010W</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ke-db3010w-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KE-DBA-AUXW</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ke-dba-auxw-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>KE-DM3010R</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ke-dm3010r-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>KE-DM3010R-KIT</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ke-dm3010r-kit-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>KE-DP3020W</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ke-dp3020w-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>KE-DP3120W</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>ke-dp3120w-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>KE-DT3001W-HAB</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ke-dt3001w-hab-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>KE-IO3101</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ke-io3101-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>KE-IO3122</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ke-io3122-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>KE-IO3144</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ke-io3144-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>NC-PF2</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>nc-pf2-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>NC-PF4</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>nc-pf4-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>NC-PF4-SC</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>nc-pf4-sc-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>NC-PF8</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>nc-pf8-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>NC-PF8-SC</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>nc-pf8-sc-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>617</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Tipo documento</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Idioma</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Subcarpeta</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Archivo</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Tamaño (KB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2X-LB</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>00-3218-501-0000-07_r007_2x-lb_installation_sheet_ml.pdf</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>00-3280-501-4003-05_r005_2x-a_series_installation_manual_en_0.pdf</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>4810</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2X-AF2-09</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>00-3280-501-4009-05_r005_2x-a_series_installation_manual_es.pdf</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>5001</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2X-AF2-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Manual usuario</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>00-3280-505-4009-04_r004_2x-a_series_operation_manual_es.pdf</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>00-3280-507-4003-03_r003_2x-a_series_quick_installation_guide_en.pdf</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2X-AF2-09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>00-3280-507-4009-03_r003_2x-a_series_quick_installation_guide_es.pdf</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2X-AF2-09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>00-3280-508-4009-03_r003_2x-a_series_quick_operation_guide_es.pdf</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>00-3280-508-4109-06_r006_2x-at_series_quick_start_guide_es.pdf</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Guía rápida</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>00-3280-508-4209-02_r002_2x-at_series_quick_operation_guide_es.pdf</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2X-A-LB</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>00-3301-501-4000-04_r004_2x-a-lb_loop_board_installation_sheet_ml.pdf</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2010-2A-PAK-HPL</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>00-3301-501-4100-04_r004_2010-2a-pak-hpl_registration_guide_ml.pdf</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>FD2705R</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0044-055-02_-_aritech_ra_-_fd2705-10r_addendum_-_en_de.pdf</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>IU2055NC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>10-5106-501-55nc-05_r005_iu2055nc_installation_sheet_ml.pdf</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AS2364</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>18-187110-10.pdf</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1608</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2010-2-PAK-RMSDK</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2010-2-pak-rmsdk-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2010-2A-PAK-HPL</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2010-2a-pak-hpl-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>FD2705R</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Manual usuario</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>22318.18.08_-_aritech_ra_-_fd2705-10r_english_std_reflective_user_guide_-_en.pdf</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2X-A-LB</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2x-a-lb-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1557</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2X-AF2-09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2x-af2-09-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2x-at-f2-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2X-LB</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2x-lb-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1556</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>3103267-en_r001_2x-a_series_kuwait_marketplace_manual.pdf</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ASW2367</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>aritech_ins570-8_combined.pdf</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>AS2363</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>as2363-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>AS2364</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>as2364-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ASW2366</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>asw2366-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ASW2367</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>asw2367-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2010-2-PAK-RMSDK</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>bcn-3100032-ml_r002_2010-2-pak-rmsdk_registration_guide.pdf</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>bcn-3100035-en_r006_2x-a_series_addressable_control_panel_compatibility_list_0.pdf</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2X-AT-F2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>bcn-3100036-en_r002_2x-a_and_zp2-a_series_addressable_control_panel_compatibility_list_900_series_protocol.pdf</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>FD2705R</t>
+        </is>
+      </c>
       <c r="B32" t="inlineStr">
         <is>
           <t>Datasheet</t>
@@ -35135,11 +36935,749 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>nc-pf8-sc-161721-es.pdf</t>
+          <t>fd2705r-62536-es.pdf</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>617</v>
+        <v>499</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FD2710R</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>fd2710r-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>IU2055NC</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>iu2055nc-62536-es.pdf</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1069</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Tipo documento</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Idioma</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Subcarpeta</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Archivo</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Tamaño (KB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FHSD8310</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>04-4001-501-2009-12_r012_modulaser_en_54-20_installation_manual_es_edwards_0.pdf</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>6021</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FHSD8310</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>fhsd8310-63296-es.pdf</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FHSD8330</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>fhsd8330-63296-es.pdf</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>462</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Tipo documento</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Idioma</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Subcarpeta</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Archivo</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Tamaño (KB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>N-MC-BB-G</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>03-0210-501-4301-02_r002_n-mc_series_mcp_backbox_installation_sheet_ml.pdf</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NC-MC-0-G</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>03-0211-501-3000-05_r005_nc_series_conventional_mcp_installation_sheet_ml_0.pdf</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>9-30441</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>04-4001-501-1700-06_r006_aritech_apic_installation_sheet_ml_0.pdf</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AD68N-0100</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Manual técnico</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>20-8501-509-dl03-04_alarmline_ii_digital_lhd_cable_technical_manual_en.pdf</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>9-10900</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>9-10900-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>9-10906</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>9-10906-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9-10908</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>9-10908-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9-10909</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>9-10909-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>9-10927</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>9-10927-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>9-10954-100</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>9-10954-100-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9-30441</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>9-30441-62576-es.pdf</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AD68N-0100</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ad68n-0100-1-es.pdf</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DM715</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>dm715-63296-es.pdf</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>N-MC-BB-G</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>n-mc-bb-g-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NC-MC-0-G</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nc-mc-0-g-161721-es.pdf</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SC010</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>sds0098es_solo_a10_iss_2.1.pdf</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
corpus(s54): Detnov CAD-171 (serie Vesta) — 5 manuales + inventario (DEC-030)
- Central Detnov nueva no identificada (CAD-171, analogica 2 lazos, serie Vesta).
- detnov.com = WordPress estatico -> 5 PDFs por links directos (datasheet ES+EN,
  instalacion MI-716, config/software CAD-250 MC-380/MS-416).
- No-duplicados verificado: la hoja Detnov ya tiene CAD-250 instalacion+usuario,
  NO config/software -> contenido nuevo. Parse 5/5 OK (~218pp/~$12).
- Inventario: APPEND a la hoja Detnov legacy (4-col; NO rebuild) -> 110 prod/124 docs.
- INERTE: ingesta a chunks_v2 DIFERIDA (gate RULER + Protocolo 3).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Inventario_Manuales.xlsx
+++ b/data/Inventario_Manuales.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -563,14 +563,14 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Ingestado en Supabase</t>
+          <t>109 ingestados en Supabase + CAD-171 (s54): parse OK, ingesta DIFERIDA</t>
         </is>
       </c>
     </row>
@@ -710,45 +710,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
@@ -763,7 +724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D122"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3175,14 +3136,114 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="5" t="inlineStr">
-        <is>
-          <t>Total: 109 productos</t>
-        </is>
-      </c>
-      <c r="B122" s="5" t="inlineStr">
-        <is>
-          <t>119 documentos</t>
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>CAD-171</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Datasheet_CAD-171-DS-736-es.pdf</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>2138</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>CAD-171</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Datasheet-CAD-171-DS-737-en.pdf</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>2149</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>CAD-171</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Manual_CAD-171-MI-716-es.pdf</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>7317</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>CAD-171</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Manual configuración</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-Configuracion-MC-380-es-2026-c.pdf</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>32329</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>CAD-171</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Manual software configuración</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-software-configuracion-MS-416-es-2026-b.pdf</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>11613</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>Total: 110 productos</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>124 documentos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
corpus(s54): Detnov CAD-171 (serie Vesta) — 5 manuales + inventario (DEC-030) (#48)
- Central Detnov nueva no identificada (CAD-171, analogica 2 lazos, serie Vesta).
- detnov.com = WordPress estatico -> 5 PDFs por links directos (datasheet ES+EN,
  instalacion MI-716, config/software CAD-250 MC-380/MS-416).
- No-duplicados verificado: la hoja Detnov ya tiene CAD-250 instalacion+usuario,
  NO config/software -> contenido nuevo. Parse 5/5 OK (~218pp/~$12).
- Inventario: APPEND a la hoja Detnov legacy (4-col; NO rebuild) -> 110 prod/124 docs.
- INERTE: ingesta a chunks_v2 DIFERIDA (gate RULER + Protocolo 3).

Co-authored-by: albertofontiber <271603099+albertofontiber@users.noreply.github.com>
Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Inventario_Manuales.xlsx
+++ b/data/Inventario_Manuales.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -563,14 +563,14 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Ingestado en Supabase</t>
+          <t>109 ingestados en Supabase + CAD-171 (s54): parse OK, ingesta DIFERIDA</t>
         </is>
       </c>
     </row>
@@ -710,45 +710,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
@@ -763,7 +724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D122"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3175,14 +3136,114 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="5" t="inlineStr">
-        <is>
-          <t>Total: 109 productos</t>
-        </is>
-      </c>
-      <c r="B122" s="5" t="inlineStr">
-        <is>
-          <t>119 documentos</t>
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>CAD-171</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Datasheet_CAD-171-DS-736-es.pdf</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>2138</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>CAD-171</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Datasheet-CAD-171-DS-737-en.pdf</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>2149</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>CAD-171</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Manual_CAD-171-MI-716-es.pdf</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>7317</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>CAD-171</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Manual configuración</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-Configuracion-MC-380-es-2026-c.pdf</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>32329</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>CAD-171</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Manual software configuración</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-software-configuracion-MS-416-es-2026-b.pdf</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>11613</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>Total: 110 productos</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>124 documentos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
corpus(s55): Detnov CAD-201 + CAD-201-PLUS (serie Vesta) — solo-no-duplicados (DEC-032)
- 2 centrales mas de la serie Vesta. detnov.com WordPress directo.
- Dedup fuerte: CAD-201 y CAD-201-PLUS linkan los mismos 5 PDFs, 2 ya teniamos
  (config/software CAD-250 de CAD-171) -> solo 3 nuevos (datasheet ES+EN +
  instalacion MI-715). CAD-201-PLUS sin docs propios.
- Parse 3/3 OK (~62pp/~$3); los 2 config saltados por SHA.
- Inventario: APPEND a hoja Detnov legacy -> 112 prod/134 docs.
- INERTE: ingesta a chunks_v2 DIFERIDA.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Inventario_Manuales.xlsx
+++ b/data/Inventario_Manuales.xlsx
@@ -563,14 +563,14 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>109 ingestados en Supabase + CAD-171 (s54): parse OK, ingesta DIFERIDA</t>
+          <t>109 ingestados en Supabase + CAD-171/201/201-PLUS (s54-55): parse OK, ingesta DIFERIDA</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3135,6 +3135,7 @@
         <v>977</v>
       </c>
     </row>
+    <row r="121"/>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
@@ -3236,14 +3237,214 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="5" t="inlineStr">
-        <is>
-          <t>Total: 110 productos</t>
-        </is>
-      </c>
-      <c r="B127" s="5" t="inlineStr">
-        <is>
-          <t>124 documentos</t>
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>CAD-201</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Datasheet_CAD-201-DS-740-es.pdf</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>6719</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>CAD-201</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Datasheet_CAD-201-DS-741-en.pdf</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>6730</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>CAD-201</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Manual_CAD-201-MI-715-es.pdf</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>8385</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>CAD-201</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Manual configuración</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-Configuracion-MC-380-es-2026-c.pdf</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>32329</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>CAD-201</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Manual software configuración</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-software-configuracion-MS-416-es-2026-b.pdf</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>11613</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>CAD-201-PLUS</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Datasheet_CAD-201-DS-740-es.pdf</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>6719</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>CAD-201-PLUS</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Datasheet_CAD-201-DS-741-en.pdf</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>6730</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>CAD-201-PLUS</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Manual_CAD-201-MI-715-es.pdf</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>8385</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>CAD-201-PLUS</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Manual configuración</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-Configuracion-MC-380-es-2026-c.pdf</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>32329</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>CAD-201-PLUS</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Manual software configuración</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-software-configuracion-MS-416-es-2026-b.pdf</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>11613</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>Total: 112 productos</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>134 documentos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
corpus(s55): Detnov CAD-201 + CAD-201-PLUS (serie Vesta) — solo-no-duplicados (DEC-032) (#50)
- 2 centrales mas de la serie Vesta. detnov.com WordPress directo.
- Dedup fuerte: CAD-201 y CAD-201-PLUS linkan los mismos 5 PDFs, 2 ya teniamos
  (config/software CAD-250 de CAD-171) -> solo 3 nuevos (datasheet ES+EN +
  instalacion MI-715). CAD-201-PLUS sin docs propios.
- Parse 3/3 OK (~62pp/~$3); los 2 config saltados por SHA.
- Inventario: APPEND a hoja Detnov legacy -> 112 prod/134 docs.
- INERTE: ingesta a chunks_v2 DIFERIDA.

Co-authored-by: albertofontiber <271603099+albertofontiber@users.noreply.github.com>
Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Inventario_Manuales.xlsx
+++ b/data/Inventario_Manuales.xlsx
@@ -563,14 +563,14 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>109 ingestados en Supabase + CAD-171 (s54): parse OK, ingesta DIFERIDA</t>
+          <t>109 ingestados en Supabase + CAD-171/201/201-PLUS (s54-55): parse OK, ingesta DIFERIDA</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3135,6 +3135,7 @@
         <v>977</v>
       </c>
     </row>
+    <row r="121"/>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
@@ -3236,14 +3237,214 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="5" t="inlineStr">
-        <is>
-          <t>Total: 110 productos</t>
-        </is>
-      </c>
-      <c r="B127" s="5" t="inlineStr">
-        <is>
-          <t>124 documentos</t>
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>CAD-201</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Datasheet_CAD-201-DS-740-es.pdf</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>6719</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>CAD-201</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Datasheet_CAD-201-DS-741-en.pdf</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>6730</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>CAD-201</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Manual_CAD-201-MI-715-es.pdf</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>8385</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>CAD-201</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Manual configuración</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-Configuracion-MC-380-es-2026-c.pdf</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>32329</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>CAD-201</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Manual software configuración</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-software-configuracion-MS-416-es-2026-b.pdf</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>11613</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>CAD-201-PLUS</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Datasheet_CAD-201-DS-740-es.pdf</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>6719</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>CAD-201-PLUS</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Datasheet_CAD-201-DS-741-en.pdf</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>6730</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>CAD-201-PLUS</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Manual instalación</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Manual_CAD-201-MI-715-es.pdf</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>8385</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>CAD-201-PLUS</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Manual configuración</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-Configuracion-MC-380-es-2026-c.pdf</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>32329</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>CAD-201-PLUS</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Manual software configuración</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>CAD-250_Manual-software-configuracion-MS-416-es-2026-b.pdf</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>11613</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>Total: 112 productos</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>134 documentos</t>
         </is>
       </c>
     </row>

</xml_diff>